<commit_message>
docs: sync ERD and API contract with what is built
- ERD: implemented status, timestamptz everywhere, username-only admins,
  anon/authenticated privileges revoked
- API contract: OFF_SITE / LOCATION_REQUIRED details (reason,
  venue_wifi_name), TOO_MANY_REQUESTS retry_after, "what can and cannot
  fool the on-site check" section
- regenerate the images and spreadsheets in docs/export

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/export/api-contract.xlsx
+++ b/docs/export/api-contract.xlsx
@@ -21,7 +21,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Requests &amp; Responses'!$A$1:$E$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Visitor flow'!$A$1:$E$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Error codes'!$A$1:$D$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'On-site access'!$A$1:$B$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'On-site access'!$A$1:$B$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Rate limits'!$A$1:$B$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Traceability'!$A$1:$B$17</definedName>
   </definedNames>
@@ -565,7 +565,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Draft for review (step 1, revision 2). Source of truth: docs/03-api-contract.md</t>
+          <t>Revision 3. Implemented so far: access-check, the on-site gate, error shape, IP-aware rate limits. Other endpoints still to be built. Source of truth: docs/03-api-contract.md</t>
         </is>
       </c>
     </row>
@@ -2155,7 +2155,11 @@
           <t>Request is outside the event's allowed IP range / geofence.</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr"/>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>details: { reason, venue_wifi_name } - show the No access page naming the Wi-Fi</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="n">
@@ -2171,7 +2175,11 @@
           <t>The event's mode needs location and lat/lng were not sent.</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr"/>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>details: { reason, venue_wifi_name }</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="n">
@@ -2351,7 +2359,11 @@
           <t>Generic throttle on any other endpoint.</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr"/>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>details.retry_after (seconds) + Retry-After header</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:D14"/>
@@ -2365,7 +2377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -2519,29 +2531,65 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Venue checklist</t>
+          <t>Not checked: the Wi-Fi name</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Public IPv4/IPv6 egress (static? one line or two?) | captive portal or proxy that rewrites client IPs? | capacity for 1,000+ simultaneous clients | can Apple Private Relay be blocked on the guest network?</t>
+          <t>A browser cannot read the network name and the API never asks. venue_wifi_name is display text only; a fake hotspot with the same name leaves through the attacker's own internet line and is rejected with OFF_SITE.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
+          <t>Cannot be faked: IP / headers</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>The source IP cannot be forged over TCP/HTTPS. A fake X-Forwarded-For header is ignored unless it comes from a trusted proxy (automated test).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Residual risk: relay through the venue</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>An accomplice on the real Wi-Fi could tunnel remote friends' traffic out through the venue IP. Deliberate setup, and each remote voter still needs their own phone + OTP. Mitigation: client isolation and VPN blocking on the guest network.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Venue checklist</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Public IPv4/IPv6 egress (static? one line or two?) | captive portal or proxy that rewrites client IPs? | capacity for 1,000+ simultaneous clients | can Apple Private Relay be blocked on the guest network?</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
           <t>Rehearsal test</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>On the venue Wi-Fi access-check must return on_site true. Switch to mobile data: false + No access page. Test iPhone and Android.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B14"/>
+  <autoFilter ref="A1:B17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
backend: Wi-Fi-only on-site rule and demo votes command
- drop events.access_mode and events.geofence; the on-site check is
  only the venue Wi-Fi public IP allowlist (allowed_cidrs)
- remove location handling and LOCATION_REQUIRED; access-check now
  returns { on_site, reason, venue_wifi_name }
- admin Event settings: rule selector and geofence fields removed
- php artisan voting:demo-votes {event} [--visitors=N] [--clear]:
  bulk-inserts demo visitors and weighted votes for the leaderboard;
  demo rows are tagged with 192.0.2.1 (RFC 5737) so --clear never
  touches real data
- docs and exports updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/export/api-contract.xlsx
+++ b/docs/export/api-contract.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Endpoints'!$A$1:$I$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Requests &amp; Responses'!$A$1:$E$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Visitor flow'!$A$1:$E$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Error codes'!$A$1:$D$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Error codes'!$A$1:$D$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'On-site access'!$A$1:$B$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Rate limits'!$A$1:$B$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Traceability'!$A$1:$B$17</definedName>
@@ -685,7 +685,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Applied on otp/request, otp/verify, votes. Decided server-side from the event's settings (access_mode ip | geo | either | both). MC2026 default = venue Wi-Fi ONLY (access_mode = ip); off-site visitors are routed to a 'No access' page. See the 'On-site access' tab.</t>
+          <t>Applied on otp/request, otp/verify, votes. Venue Wi-Fi ONLY: the client's public IP must be in the event's allowed_cidrs; off-site visitors are routed to a 'No access' page. See the 'On-site access' tab.</t>
         </is>
       </c>
     </row>
@@ -913,7 +913,7 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Is this device on-site? Drives the 'No access' page (optional query: lat, lng)</t>
+          <t>Is this device on the venue Wi-Fi? Drives the 'No access' page</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -1018,7 +1018,7 @@
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>EVENT_NOT_FOUND, VALIDATION_FAILED, OFF_SITE, LOCATION_REQUIRED, VOTING_CLOSED, OTP_RATE_LIMITED</t>
+          <t>EVENT_NOT_FOUND, VALIDATION_FAILED, OFF_SITE, VOTING_CLOSED, OTP_RATE_LIMITED</t>
         </is>
       </c>
     </row>
@@ -1063,7 +1063,7 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>EVENT_NOT_FOUND, VALIDATION_FAILED, OFF_SITE, LOCATION_REQUIRED, OTP_INVALID, OTP_EXPIRED, TOO_MANY_REQUESTS</t>
+          <t>EVENT_NOT_FOUND, VALIDATION_FAILED, OFF_SITE, OTP_INVALID, OTP_EXPIRED, TOO_MANY_REQUESTS</t>
         </is>
       </c>
     </row>
@@ -1198,7 +1198,7 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>UNAUTHENTICATED, OFF_SITE, LOCATION_REQUIRED, VOTING_CLOSED, UNVERIFIED, VALIDATION_FAILED, INVALID_EXHIBITOR_FOR_CATEGORY, ALREADY_VOTED, TOO_MANY_REQUESTS</t>
+          <t>UNAUTHENTICATED, OFF_SITE, VOTING_CLOSED, UNVERIFIED, VALIDATION_FAILED, INVALID_EXHIBITOR_FOR_CATEGORY, ALREADY_VOTED, TOO_MANY_REQUESTS</t>
         </is>
       </c>
     </row>
@@ -1427,7 +1427,7 @@
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>Query (optional): lat, lng</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
@@ -1435,8 +1435,6 @@
           <t>{
   "data": {
     "on_site": false,
-    "mode": "ip",
-    "requires_location": false,
     "reason": "OUTSIDE_IP_RANGE",
     "venue_wifi_name": "MC2026-Guest"
   }
@@ -1445,7 +1443,7 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>If on_site is false -&gt; route to the 'No access' page: 'Connect to {venue_wifi_name} and try again' + a Try again button that calls this endpoint again. reason: null | OUTSIDE_IP_RANGE | OUTSIDE_GEOFENCE | LOCATION_REQUIRED. If requires_location is true (geofence modes only), ask the browser for geolocation and send lat/lng on write calls. The redirect is UX only - the API re-checks on every write endpoint.</t>
+          <t>If on_site is false -&gt; route to the 'No access' page: 'Connect to {venue_wifi_name} and try again' + a Try again button that calls this endpoint again. reason: null | OUTSIDE_IP_RANGE. The redirect is UX only - the API re-checks on every write endpoint.</t>
         </is>
       </c>
     </row>
@@ -1520,7 +1518,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>full_name 2-80 chars. phone in any common format; normalised to E.164 = the visitor's UID (0791234567 and +962791234567 are the same visitor). lat/lng only when requires_location is true (geofence modes - not needed for the default Wi-Fi-only rule). Verification is PER EVENT: this runs again for every new event, even if the phone was verified for another one. Same response whether or not the phone was seen before (no enumeration).</t>
+          <t>full_name 2-80 chars. phone in any common format; normalised to E.164 = the visitor's UID (0791234567 and +962791234567 are the same visitor). Verification is PER EVENT: this runs again for every new event, even if the phone was verified for another one. Same response whether or not the phone was seen before (no enumeration).</t>
         </is>
       </c>
     </row>
@@ -1641,9 +1639,7 @@
         <is>
           <t>{
   "category_id": 1,
-  "exhibitor_id": 12,
-  "lat": 31.9539,
-  "lng": 35.9106
+  "exhibitor_id": 12
 }</t>
         </is>
       </c>
@@ -1839,7 +1835,7 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Check voting state and location</t>
+          <t>Check voting state and Wi-Fi</t>
         </is>
       </c>
       <c r="D3" s="8" t="inlineStr">
@@ -1849,7 +1845,7 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>on_site false -&gt; 'No access' page (join {venue_wifi_name}, Try again). Voting closed -&gt; closed message. Ask for geolocation only if requires_location</t>
+          <t>on_site false -&gt; 'No access' page (join {venue_wifi_name}, Try again). Voting closed -&gt; closed message.</t>
         </is>
       </c>
     </row>
@@ -2090,7 +2086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2152,7 +2148,7 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Request is outside the event's allowed IP range / geofence.</t>
+          <t>Request is not coming from the event's venue Wi-Fi (public IP outside allowed_cidrs).</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
@@ -2167,17 +2163,17 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>LOCATION_REQUIRED</t>
+          <t>VOTING_CLOSED</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>The event's mode needs location and lat/lng were not sent.</t>
+          <t>Voting is not currently open for this event.</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>details: { reason, venue_wifi_name }</t>
+          <t>details.status: closed | scheduled</t>
         </is>
       </c>
     </row>
@@ -2187,69 +2183,69 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>VOTING_CLOSED</t>
+          <t>UNVERIFIED</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Voting is not currently open for this event.</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>details.status: closed | scheduled</t>
-        </is>
-      </c>
+          <t>Visitor's registration for this event is not verified (defensive; should not occur).</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="n">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>UNVERIFIED</t>
+          <t>EVENT_NOT_FOUND</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Visitor's registration for this event is not verified (defensive; should not occur).</t>
+          <t>Unknown or inactive event slug.</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="n">
-        <v>404</v>
+        <v>409</v>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>EVENT_NOT_FOUND</t>
+          <t>ALREADY_VOTED</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Unknown or inactive event slug.</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr"/>
+          <t>Already voted in this category for a different exhibitor.</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>details: { category_id, exhibitor_id } = the vote already held</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="n">
-        <v>409</v>
+        <v>422</v>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>ALREADY_VOTED</t>
+          <t>VALIDATION_FAILED</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Already voted in this category for a different exhibitor.</t>
+          <t>Field errors.</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>details: { category_id, exhibitor_id } = the vote already held</t>
+          <t>details.fields</t>
         </is>
       </c>
     </row>
@@ -2259,19 +2255,15 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>VALIDATION_FAILED</t>
+          <t>INVALID_EXHIBITOR_FOR_CATEGORY</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Field errors.</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>details.fields</t>
-        </is>
-      </c>
+          <t>Exhibitor is not entered in that category of this event (or is inactive).</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="n">
@@ -2279,15 +2271,19 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>INVALID_EXHIBITOR_FOR_CATEGORY</t>
+          <t>OTP_INVALID</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Exhibitor is not entered in that category of this event (or is inactive).</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr"/>
+          <t>Wrong code.</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>details.attempts_remaining</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="n">
@@ -2295,35 +2291,35 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>OTP_INVALID</t>
+          <t>OTP_EXPIRED</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Wrong code.</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>details.attempts_remaining</t>
-        </is>
-      </c>
+          <t>Code expired, consumed, or attempts exhausted - request a new one.</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="n">
-        <v>422</v>
+        <v>429</v>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>OTP_EXPIRED</t>
+          <t>OTP_RATE_LIMITED</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Code expired, consumed, or attempts exhausted - request a new one.</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr"/>
+          <t>Too many OTP requests.</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>details.retry_after (seconds) + Retry-After header</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="n">
@@ -2331,12 +2327,12 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>OTP_RATE_LIMITED</t>
+          <t>TOO_MANY_REQUESTS</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Too many OTP requests.</t>
+          <t>Generic throttle on any other endpoint.</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -2345,28 +2341,8 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="6" t="n">
-        <v>429</v>
-      </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>TOO_MANY_REQUESTS</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Generic throttle on any other endpoint.</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>details.retry_after (seconds) + Retry-After header</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:D14"/>
+  <autoFilter ref="A1:D13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2399,12 +2375,12 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>MC2026 default: venue Wi-Fi ONLY</t>
+          <t>Rule: venue Wi-Fi ONLY</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>access_mode = ip, geofence off. allowed_cidrs = the venue Wi-Fi's public egress ranges (IPv4 AND IPv6). All visitors behind the Wi-Fi NAT share these addresses. A client cannot forge its public IP, unlike GPS, so this is the fairest rule against remote voting.</t>
+          <t>No location/GPS check. allowed_cidrs = the venue Wi-Fi's public egress ranges (IPv4 AND IPv6). All visitors behind the Wi-Fi NAT share these addresses. A client cannot forge its public IP, unlike GPS, so this is the fairest rule against remote voting.</t>
         </is>
       </c>
     </row>
@@ -2416,7 +2392,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>A visitor who cannot join the Wi-Fi (overload, VPN, Private Relay, phone problem) cannot vote. Mitigations: Wi-Fi sized for 1,000+ clients, signage with the network name, troubleshooting steps on the No access page, and the Makerspace can relax access_mode LIVE in the admin panel (e.g. to 'either') if Wi-Fi problems appear on the day.</t>
+          <t>A visitor who cannot join the Wi-Fi (overload, VPN, Private Relay, phone problem) cannot vote. Mitigations: Wi-Fi sized for 1,000+ clients, signage with the network name, troubleshooting steps on the No access page, and admins can add IP ranges LIVE in Event settings (e.g. a backup internet line).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
backend: TV results API, live stream and display tokens
- GET /events/{event}/results and /results/stream (Server-Sent Events):
  full snapshot on connect and on change, heartbeat, closes after ~5 min
  or on token revoke; standings cached ~1 s; voting status included
- Display tokens owned by the event (results:read + event:<id>), accepted
  from the Authorization header or ?token=; throttled per token and IP,
  not tied to the venue Wi-Fi
- Admin "TV displays" page: create (shown once, 1/7/30-day expiry),
  last seen, revoke; audit-logged
- ApiError responses are no longer reported to laravel.log
- voting:demo-votes: every demo visitor votes at least once (fixes a
  flaky test)
- Docs: API contract rev 4 (results section, rate limits), ERD tokens,
  regenerated api-contract exports

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/export/api-contract.xlsx
+++ b/docs/export/api-contract.xlsx
@@ -22,7 +22,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Visitor flow'!$A$1:$E$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Error codes'!$A$1:$D$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'On-site access'!$A$1:$B$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Rate limits'!$A$1:$B$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Rate limits'!$A$1:$B$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Traceability'!$A$1:$B$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -565,7 +565,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Revision 3. Implemented: every visitor endpoint (events, event, categories, access-check, OTP request/verify, me, logout, votes), error shape, rate limits. Until the SMS gateway is connected, codes go to backend/storage/logs/sms.log. Still to build: results + results/stream (TV). Source of truth: docs/03-api-contract.md</t>
+          <t>Revision 4. Every endpoint is implemented: visitor endpoints (events, event, categories, access-check, OTP request/verify, me, logout, votes) and TV endpoints (results, results/stream), error shape, rate limits. Display tokens: admin panel &gt; TV displays. Until the SMS gateway is connected, codes go to backend/storage/logs/sms.log. Source of truth: docs/03-api-contract.md</t>
         </is>
       </c>
     </row>
@@ -1675,7 +1675,7 @@
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Header: Authorization: Bearer &lt;display token&gt; (or ?token=)</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
@@ -1711,14 +1711,19 @@
           }
         ]
       }
-    ]
+    ],
+    "voting": {
+      "status": "open",
+      "opens_at": null,
+      "closes_at": "2026-11-14T18:00:00Z"
+    }
   }
 }</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Ties share a rank (1, 1, 3). Every active exhibitor appears, including those with 0 votes. total_voters = distinct visitors with at least one vote in this event. Cached ~1 s server-side.</t>
+          <t>Ties share a rank (1, 1, 3). Every active exhibitor appears, including those with 0 votes. total_voters = distinct visitors with at least one vote in this event. voting = same object as GET /events/{event}. Cached ~1 s server-side. No on-site gate: the TV may be on any network. Display tokens are created in the admin panel (TV displays), shown once, expire after 1/7/30 days, revocable.</t>
         </is>
       </c>
     </row>
@@ -1740,13 +1745,13 @@
         <is>
           <t>retry: 3000
 event: snapshot
-data: {"event":{…},"generated_at":"…","total_voters":412,"total_votes":1190,"categories":[…]}
+data: {"event":{…},"generated_at":"…","total_voters":412,"total_votes":1190,"categories":[…],"voting":{…}}
 : heartbeat</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Full snapshot (same JSON as /results data) on connect and whenever tallies change (checked ~2 s); heartbeat comment ~15 s; browser auto-reconnects (retry 3000) - no catch-up logic needed. EventSource cannot set headers, hence ?token=. Fallback: poll GET /results every 2-3 s.</t>
+          <t>Full snapshot (same JSON as /results data) on connect and whenever tallies or voting status change (checked ~2 s); heartbeat comment after ~15 s with no change. The server closes the stream after ~5 min, on token revoke or event deactivation; the browser auto-reconnects (retry 3000) - no catch-up logic needed. EventSource cannot set headers, hence ?token=. EventSource does not retry a 401: on onerror with readyState CLOSED show 'display token invalid'. Fallback: poll GET /results every 2-3 s.</t>
         </is>
       </c>
     </row>
@@ -2133,7 +2138,7 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>details.reason: missing | invalid | expired | wrong_event - send the visitor through the OTP flow for this event</t>
+          <t>details.reason: missing | invalid | expired | wrong_event - visitor: run the OTP flow for this event; TV: show 'display token invalid'</t>
         </is>
       </c>
     </row>
@@ -2576,7 +2581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -2658,29 +2663,41 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Venue IPs (inside allowed_cidrs)</t>
+          <t>GET .../results, .../results/stream (TV)</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>NO per-IP throttle; only a safety ceiling of 5,000 requests / min per IP to stop a runaway script</t>
+          <t>120 / min per display token + 600 / min per IP. Not tied to the venue Wi-Fi (a screen may be on another network)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
+          <t>Venue IPs (inside allowed_cidrs)</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>NO per-IP throttle; only a safety ceiling of 5,000 requests / min per IP to stop a runaway script</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
           <t>Off-site IPs (outside allowed_cidrs)</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>30 / min per IP on every endpoint (they are rejected by the gate anyway)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B8"/>
+  <autoFilter ref="A1:B9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>